<commit_message>
As-built three-core spec cut to one page: wire column gives the current the vendor's wire can carry at 4.5 A/mm2, bobbin and core pictures drawn after the vendor's, notes removed
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3H8Na8buSZY2uPpuuSkn7
</commit_message>
<xml_diff>
--- a/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_asbuilt.xlsx
+++ b/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_asbuilt.xlsx
@@ -87,17 +87,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -174,6 +175,61 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1819275"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3143250" cy="3648075"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -465,36 +521,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TRANSFORMER SPECIFICATION — as built (3코어 시험 보드)</t>
+          <t>TRANSFORMER SPECIFICATION — as built</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>L6790A single-stage PF LLC, 25 V / 26.3 A.  세트 권선비 7.5 : 1 = 유닛 5 : 2 × 3개(1차 직렬, 2차 병렬).  아래 값은 전부 유닛 하나 기준.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>L6790A single-stage PF LLC, 25 V / 26.3 A.  3 units per set (primaries in series, secondaries in parallel).  Values per unit.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>1.  WINDING  (단자 번호는 벤더 보빈 번호: 4핀 쪽 1–4, 8핀 쪽 5–12)</t>
+          <t>1.  WINDING</t>
         </is>
       </c>
     </row>
@@ -526,7 +581,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Current  rms / peak</t>
+          <t>Current capability (4.5 A/mm²)</t>
         </is>
       </c>
     </row>
@@ -551,12 +606,12 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Litz 0.1 mm × 130</t>
+          <t>Litz 0.1 mm × 130  (1.02 mm²)</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>10.9 A   /   18.3 A</t>
+          <t>4.6 A rms</t>
         </is>
       </c>
     </row>
@@ -581,12 +636,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Litz 0.1 mm × 110, NS3 과 bifilar</t>
+          <t>Litz 0.1 mm × 110, bifilar  (0.86 mm²)</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>9.4 A   /   32.9 A</t>
+          <t>3.9 A rms</t>
         </is>
       </c>
     </row>
@@ -611,12 +666,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Litz 0.1 mm × 110, NS2 와 bifilar</t>
+          <t>Litz 0.1 mm × 110, bifilar  (0.86 mm²)</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>9.4 A   /   32.9 A</t>
+          <t>3.9 A rms</t>
         </is>
       </c>
     </row>
@@ -626,7 +681,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>NAUX  Auxiliary (VCC, ZCD)</t>
+          <t>NAUX  Auxiliary</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -641,27 +696,26 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>ø0.4 mm</t>
+          <t>ø0.4 mm  (0.126 mm²)</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>104 mA dc load (VCC)</t>
+          <t>0.57 A rms</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>센터탭은 보드에서 만든다(트랜스포머 안에서 잇지 않는다). 어느 두 핀을 이을지는 4절의 극성 시험으로 정한다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11"/>
+          <t>Centre tap on the PCB: the NS2 end and the NS3 start that add up (section 4). Not joined inside the transformer.</t>
+        </is>
+      </c>
+    </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2.  ELECTRICAL REQUIREMENTS  (LCR 100 kHz / 1 V, 직렬 등가 L_s, OPEN/SHORT 보정, 유닛마다)</t>
+          <t>2.  ELECTRICAL REQUIREMENTS   (LCR 100 kHz / 1 V, series L_s, per unit)</t>
         </is>
       </c>
     </row>
@@ -681,19 +735,15 @@
           <t>Terminal</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>Condition</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Note</t>
         </is>
       </c>
     </row>
@@ -711,19 +761,15 @@
           <t>1 – 4</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>10.33 µH    ±10 %</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>다른 권선 전부 OPEN</t>
-        </is>
-      </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>L_m + L_leak.  3개 직렬이면 합 ≈ 31 µH</t>
+          <t>all other windings OPEN</t>
         </is>
       </c>
     </row>
@@ -741,19 +787,15 @@
           <t>1 – 4</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr"/>
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>3.67 µH    ±10 %</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>2차 둘 다 SHORT (5–9 와 7–11), NAUX OPEN</t>
-        </is>
-      </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>공진 인덕터 L_r 의 1/3.  목표값이지 최대값이 아니다.  3개 직렬이면 합 ≈ 11 µH</t>
+          <t>5–9 and 7–11 both SHORT, 2–3 OPEN</t>
         </is>
       </c>
     </row>
@@ -765,7 +807,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>반쪽 누설 (기록)</t>
+          <t>Leakage, one half</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -773,19 +815,15 @@
           <t>1 – 4</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>기록</t>
-        </is>
-      </c>
+      <c r="D16" s="5" t="inlineStr"/>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>5–9 만 SHORT, 다음 7–11 만 SHORT</t>
+          <t>record</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>2번과 몇 % 안이면 bifilar 정상.  크게 높으면 그 값이 탱크가 보는 L_r</t>
+          <t>5–9 only SHORT, then 7–11 only SHORT</t>
         </is>
       </c>
     </row>
@@ -803,84 +841,70 @@
           <t>1 – 4</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>초기 인덕턴스의 ≥ 90 %</t>
-        </is>
-      </c>
+      <c r="D17" s="5" t="inlineStr"/>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>시험 전류 16 A, 상온, 다른 권선 OPEN</t>
+          <t>≥ 90 % of initial inductance</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>벤더 사본의 15 A 는 옛 값.  16 A 로 재면 둘 다 덮는다</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>D.C RESISTANCE</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>1–4 / 5–9 / 7–11</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>기록</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>4단자 측정</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>동손 추정에 쓴다</t>
+          <t>16 A dc, room temperature, other windings OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>3.  CORE   (A_e 114 mm², l_e 58.82 mm, V_e 6706 mm³, C1 0.52 mm⁻¹, ≈ 33.8 g/pair, material: TBD)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>3.  CORE  (벤더 도면)</t>
+      <c r="A20" s="5" t="inlineStr"/>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>42.00 ± 0.60</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>6.00 ± 0.20</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr"/>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Dimension</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Value (mm)</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Effective parameter</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Check</t>
+      <c r="A21" s="5" t="inlineStr"/>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>7.85 ± 0.15</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr"/>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>4.85 ± 0.15</t>
         </is>
       </c>
     </row>
@@ -888,27 +912,23 @@
       <c r="A22" s="5" t="inlineStr"/>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>42.00 ± 0.60</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>A_e</t>
-        </is>
-      </c>
+          <t>19.00 ± 0.30</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr"/>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>114 mm²</t>
+          <t>B − F</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>E × C = 6 × 19 = 114 ✓.  요구 Ae  ≥  103 mm²</t>
+          <t>3.00 ± 0.15</t>
         </is>
       </c>
     </row>
@@ -916,135 +936,29 @@
       <c r="A23" s="5" t="inlineStr"/>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>7.85 ± 0.15</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>l_e</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>58.82 mm</t>
-        </is>
-      </c>
+          <t>36.00 +0.5 / −0.3</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="5" t="inlineStr"/>
       <c r="F23" s="5" t="inlineStr"/>
     </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr"/>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>19.00 ± 0.30</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>V_e</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>6706 mm³</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>A_e × l_e = 6706 ✓</t>
-        </is>
-      </c>
-    </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr"/>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>36.00 +0.5 / −0.3</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>0.52 mm⁻¹</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>l_e / A_e = 0.516 ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr"/>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>6.00 ± 0.20</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>바깥다리</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>(A − D)/2 = 3.0 mm</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>2 × 3 × 19 = 114 = 중앙다리 ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr"/>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>4.85 ± 0.15</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>재질</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>도면에 없음 — 100 °C 의 B_s 확인</t>
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>4.  POLARITY  (before fitting)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="46" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Drive 1–4 with ~5 V, 50–100 kHz sine. 5–9 and 7–11 read 2/5 of it, 2–3 reads 1/5. Join one end of NS2 to one end of NS3 and find the pair whose remaining ends read double: those two pins are the centre tap. Near zero = wrong pair.</t>
         </is>
       </c>
     </row>
@@ -1052,123 +966,33 @@
       <c r="A28" s="5" t="inlineStr"/>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>B − F</t>
+          <t>Switching frequency</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>3.00 ± 0.15</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>무게</t>
-        </is>
-      </c>
+          <t>92  to  249 kHz</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr"/>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>≈ 33.8 g / pair</t>
+          <t>at full load</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr"/>
     </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>4.  POLARITY / CENTRE TAP  (보드에 꽂기 전에)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="50" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>1–4 에 50 ~ 100 kHz 정현파 약 5 V 를 걸고 5–9, 7–11 을 읽는다: 각각 1차의 2/5, 2–3 은 1/5.  그 다음 NS2 의 한 끝과 NS3 의 한 끝을 이어, 나머지 두 끝 사이가 반쪽의 두 배가 되는 짝을 찾는다.  그 두 핀이 센터탭이다.  0 근처면 반대 짝.  잘못 이으면 두 반쪽이 상쇄되어 출력이 없거나 단락이다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>5.  OPERATING CONDITIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr"/>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>Switching frequency</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>92  to  249 kHz</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>at full load</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr"/>
-      <c r="F34" s="5" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr"/>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>Set</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>3 units: 1차 1–4 직렬, 2차 병렬</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr"/>
-      <c r="E35" s="5" t="inlineStr"/>
-      <c r="F35" s="5" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr"/>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>Insulation</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>1차(NP1, NAUX) ↔ 2차 강화 절연</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>26OP-LM83W 승인원 4-4 · 4-5 와 같은 시험</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr"/>
-      <c r="F36" s="5" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>값의 출처: Transformer_Spec_7p5to1.xlsx(옛 3코어 설계점, 2026-10-01 상태) · 벤더가 적어 보낸 핀 · 와이어 · 코어 도면(2026-10-07).</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A38:F38"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A33:F33"/>
+  <mergeCells count="6">
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
As-built spec: bobbin picture redrawn after the vendor's side view (8-pin block with slots and boss, flanges, tube, 4-pin block with feet); spec builder saved as asbuilt_spec.py
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3H8Na8buSZY2uPpuuSkn7
</commit_message>
<xml_diff>
--- a/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_asbuilt.xlsx
+++ b/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_asbuilt.xlsx
@@ -186,7 +186,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2857500" cy="1819275"/>
+    <ext cx="2476500" cy="2600325"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -208,7 +208,7 @@
     <from>
       <col>7</col>
       <colOff>0</colOff>
-      <row>15</row>
+      <row>19</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="3143250" cy="3648075"/>

</xml_diff>

<commit_message>
As-built transformer spec: add the bench-measured column (open 10.3 uH, leakage 1.9/2.0/1.8 uH) and set values
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3H8Na8buSZY2uPpuuSkn7
</commit_message>
<xml_diff>
--- a/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_asbuilt.xlsx
+++ b/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_asbuilt.xlsx
@@ -87,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -97,6 +97,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -521,13 +524,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
   </cols>
@@ -535,7 +538,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TRANSFORMER SPECIFICATION — as built</t>
+          <t>TRANSFORMER SPECIFICATION — as built, with bench measurement</t>
         </is>
       </c>
     </row>
@@ -735,7 +738,11 @@
           <t>Terminal</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr"/>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Measured (3 units)</t>
+        </is>
+      </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Requirement</t>
@@ -761,7 +768,11 @@
           <t>1 – 4</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr"/>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>10.3 / 10.3 / 10.3 µH</t>
+        </is>
+      </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
           <t>10.33 µH    ±10 %</t>
@@ -787,7 +798,11 @@
           <t>1 – 4</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr"/>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>1.9 / 2.0 / 1.8 µH</t>
+        </is>
+      </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
           <t>3.67 µH    ±10 %</t>
@@ -815,7 +830,11 @@
           <t>1 – 4</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr"/>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>2.0 µH (one unit; 1.8 both SHORT)</t>
+        </is>
+      </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
           <t>record</t>
@@ -841,7 +860,11 @@
           <t>1 – 4</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr"/>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>not measured</t>
+        </is>
+      </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
           <t>≥ 90 % of initial inductance</t>
@@ -853,34 +876,17 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Measured 2026-10-09.  Set of 3 in series: L_r 5.7 µH (sum of leakage), L_m 25.2 µH (open 30.9 − L_r), n_eff = 7.5 / √(1 + L_r/L_m) = 6.773.  Leakage is about half the requirement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>3.  CORE   (A_e 114 mm², l_e 58.82 mm, V_e 6706 mm³, C1 0.52 mm⁻¹, ≈ 33.8 g/pair, material: TBD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr"/>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>42.00 ± 0.60</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr"/>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>6.00 ± 0.20</t>
         </is>
       </c>
     </row>
@@ -888,23 +894,23 @@
       <c r="A21" s="5" t="inlineStr"/>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>7.85 ± 0.15</t>
+          <t>42.00 ± 0.60</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr"/>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>4.85 ± 0.15</t>
+          <t>6.00 ± 0.20</t>
         </is>
       </c>
     </row>
@@ -912,23 +918,23 @@
       <c r="A22" s="5" t="inlineStr"/>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>19.00 ± 0.30</t>
+          <t>7.85 ± 0.15</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr"/>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>B − F</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>3.00 ± 0.15</t>
+          <t>4.85 ± 0.15</t>
         </is>
       </c>
     </row>
@@ -936,60 +942,85 @@
       <c r="A23" s="5" t="inlineStr"/>
       <c r="B23" s="5" t="inlineStr">
         <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>19.00 ± 0.30</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>B − F</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>3.00 ± 0.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr"/>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>36.00 +0.5 / −0.3</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr"/>
-      <c r="E23" s="5" t="inlineStr"/>
-      <c r="F23" s="5" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="5" t="inlineStr"/>
+      <c r="F24" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>4.  POLARITY  (before fitting)</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="46" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
+    <row r="27" ht="46" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Drive 1–4 with ~5 V, 50–100 kHz sine. 5–9 and 7–11 read 2/5 of it, 2–3 reads 1/5. Join one end of NS2 to one end of NS3 and find the pair whose remaining ends read double: those two pins are the centre tap. Near zero = wrong pair.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr"/>
-      <c r="B28" s="5" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr"/>
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>Switching frequency</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>92  to  249 kHz</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr"/>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>at full load</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr"/>
+      <c r="D29" s="5" t="inlineStr"/>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>at full load, design tank (L_r 11 µH)</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A18:F18"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A20:F20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
As-built spec: measured column per unit only, half-short item removed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3H8Na8buSZY2uPpuuSkn7
</commit_message>
<xml_diff>
--- a/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_asbuilt.xlsx
+++ b/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_asbuilt.xlsx
@@ -87,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -97,9 +97,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -524,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -740,7 +737,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Measured (3 units)</t>
+          <t>Measured (per unit)</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -770,7 +767,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>10.3 / 10.3 / 10.3 µH</t>
+          <t>10.3 µH</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -800,7 +797,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>1.9 / 2.0 / 1.8 µH</t>
+          <t>1.9 µH  (1.8 – 2.0)</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -815,14 +812,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>2a</t>
-        </is>
+      <c r="A16" s="5" t="n">
+        <v>3</v>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Leakage, one half</t>
+          <t>D.C OVERLAP</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -832,61 +827,72 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>2.0 µH (one unit; 1.8 both SHORT)</t>
+          <t>not measured</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>record</t>
+          <t>≥ 90 % of initial inductance</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>5–9 only SHORT, then 7–11 only SHORT</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>D.C OVERLAP</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>1 – 4</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>not measured</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>≥ 90 % of initial inductance</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
           <t>16 A dc, room temperature, other windings OPEN</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Measured 2026-10-09.  Set of 3 in series: L_r 5.7 µH (sum of leakage), L_m 25.2 µH (open 30.9 − L_r), n_eff = 7.5 / √(1 + L_r/L_m) = 6.773.  Leakage is about half the requirement.</t>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>3.  CORE   (A_e 114 mm², l_e 58.82 mm, V_e 6706 mm³, C1 0.52 mm⁻¹, ≈ 33.8 g/pair, material: TBD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr"/>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>42.00 ± 0.60</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr"/>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>6.00 ± 0.20</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>3.  CORE   (A_e 114 mm², l_e 58.82 mm, V_e 6706 mm³, C1 0.52 mm⁻¹, ≈ 33.8 g/pair, material: TBD)</t>
+      <c r="A20" s="5" t="inlineStr"/>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>7.85 ± 0.15</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>4.85 ± 0.15</t>
         </is>
       </c>
     </row>
@@ -894,23 +900,23 @@
       <c r="A21" s="5" t="inlineStr"/>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>42.00 ± 0.60</t>
+          <t>19.00 ± 0.30</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr"/>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B − F</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>6.00 ± 0.20</t>
+          <t>3.00 ± 0.15</t>
         </is>
       </c>
     </row>
@@ -918,109 +924,60 @@
       <c r="A22" s="5" t="inlineStr"/>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>7.85 ± 0.15</t>
+          <t>36.00 +0.5 / −0.3</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr"/>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>4.85 ± 0.15</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr"/>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>19.00 ± 0.30</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr"/>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>B − F</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>3.00 ± 0.15</t>
-        </is>
-      </c>
+      <c r="E22" s="5" t="inlineStr"/>
+      <c r="F22" s="5" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr"/>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>36.00 +0.5 / −0.3</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr"/>
-      <c r="E24" s="5" t="inlineStr"/>
-      <c r="F24" s="5" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>4.  POLARITY  (before fitting)</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="46" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
+    <row r="25" ht="46" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Drive 1–4 with ~5 V, 50–100 kHz sine. 5–9 and 7–11 read 2/5 of it, 2–3 reads 1/5. Join one end of NS2 to one end of NS3 and find the pair whose remaining ends read double: those two pins are the centre tap. Near zero = wrong pair.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr"/>
-      <c r="B29" s="5" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr"/>
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>Switching frequency</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>92  to  249 kHz</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr"/>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr"/>
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>at full load, design tank (L_r 11 µH)</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr"/>
+      <c r="F27" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="6">
+    <mergeCell ref="A24:F24"/>
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A26:F26"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>